<commit_message>
03/05/2025 19:16 Changed sheet name in Excel Workbook
</commit_message>
<xml_diff>
--- a/Store Data.xlsx
+++ b/Store Data.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\topna\OneDrive\Desktop\All\Unedited Power BI Recordings\Project 1 Power BI Course\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\Sales_Data_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B6C013-83BD-42F3-946D-14DB71A98126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{429760A4-2707-4625-97A9-107837F0A107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12240" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dim Customers" sheetId="1" r:id="rId1"/>
     <sheet name="Dim Product" sheetId="2" r:id="rId2"/>
     <sheet name="Dim Promotion " sheetId="3" r:id="rId3"/>
-    <sheet name="Sheet3" sheetId="4" r:id="rId4"/>
+    <sheet name="Facts Table" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>

</xml_diff>